<commit_message>
feat: live_pure task_list 17번 거래처분석에 적요 열 추가
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/journal_analyzer/live_pure/task_list_live_pure.xlsx
+++ b/journal_analyzer/live_pure/task_list_live_pure.xlsx
@@ -1,33 +1,33 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="16220" tabRatio="600" firstSheet="3" activeTab="10" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="16220" tabRatio="600" firstSheet="10" activeTab="11" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="settings" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="작성가이드" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="분석목록" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="02_거래처 전기_당기 비교" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="03_벤포드 분석" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="08_상대계정 분석" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="10_라운드넘버 분석" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="11_특수관계자 분석" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="13_매출 vs 비용 교차" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="14_심층분석 (계정별 Top) " sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="15_감사샘플링" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="17_거래처분석" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="20_잔액증감분석 (계정별 거래처별)" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="21_총계정원장" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="22_은행조회서 완전성" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="23_계정별 상세거래내역" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="24_리스완전성" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="25_손익월별분석" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="26_AI계정별분석_실행" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="27_감가상각_평가손익분석" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet name="감가상각_유형자산롤포워드" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet name="유형자산_처분손익" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="settings" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="작성가이드" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="분석목록" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_거래처 전기_당기 비교" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_벤포드 분석" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08_상대계정 분석" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_라운드넘버 분석" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_특수관계자 분석" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13_매출 vs 비용 교차" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14_심층분석 (계정별 Top) " sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15_감사샘플링" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="17_거래처분석" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="20_잔액증감분석 (계정별 거래처별)" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="21_총계정원장" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="22_은행조회서 완전성" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="23_계정별 상세거래내역" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="24_리스완전성" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="25_손익월별분석" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="26_AI계정별분석_실행" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="27_감가상각_평가손익분석" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="감가상각_유형자산롤포워드" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="유형자산_처분손익" sheetId="22" state="visible" r:id="rId22"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -39,7 +39,7 @@
   <numFmts count="3">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;_-;_-@_-"/>
-    <numFmt numFmtId="166" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="166" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
   <fonts count="7">
     <font>
@@ -71,16 +71,27 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="맑은 고딕"/>
+      <charset val="129"/>
+      <family val="3"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
       <sz val="11"/>
     </font>
     <font>
+      <name val="맑은 고딕"/>
+      <charset val="129"/>
+      <family val="3"/>
       <b val="1"/>
-      <color rgb="00305496"/>
+      <color rgb="FF305496"/>
+      <sz val="11"/>
     </font>
     <font>
-      <color rgb="00404040"/>
+      <name val="맑은 고딕"/>
+      <charset val="129"/>
+      <family val="3"/>
+      <color rgb="FF404040"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="3">
@@ -92,7 +103,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00305496"/>
+        <fgColor rgb="FF305496"/>
       </patternFill>
     </fill>
   </fills>
@@ -111,15 +122,13 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -128,6 +137,9 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="표준" xfId="0" builtinId="0"/>
@@ -264,7 +276,6 @@
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>감사자동화</author>
-    <author>tc={1816917C-A7C8-4BDA-A2E7-0DF136859404}</author>
   </authors>
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0">
@@ -284,30 +295,27 @@
     </comment>
     <comment ref="D1" authorId="0" shapeId="0">
       <text>
-        <t>차변/대변/both 중 하나 — 상세내역·월별합산에 포함할 금액 방향. 공란이면 자동으로 both(차변+대변 모두) 처리됨</t>
+        <t>원장 적요에 포함된 문구(부분일치), 콤마(,)로 여러 개 지정 가능(OR). 기재하면 계정과목·거래처명·금액열 조건에 더해 적요 조건까지 만족하는 거래만 추출. 공란이면 적요 조건 없이 기존처럼 추출. 거래처명을 비우고 적요만 적으면 적요 기준으로 추출(거래처별 시트는 적요 문구별로 생성)</t>
       </text>
     </comment>
     <comment ref="E1" authorId="0" shapeId="0">
       <text>
-        <t>Y(또는 O)로 표시한 행만 분석에 포함됨</t>
+        <t>차변/대변/both 중 하나 — 상세내역·월별합산에 포함할 금액 방향. 공란이면 자동으로 both(차변+대변 모두) 처리됨</t>
       </text>
     </comment>
     <comment ref="F1" authorId="0" shapeId="0">
       <text>
-        <t>Y로 지정하면 이 작업의 월별합산 결과를 전표관리단위(본사/2공장 등)별로도 나눠서 함께 추출 (공란=기존처럼 단위 구분 없이 합산)</t>
+        <t>Y(또는 O)로 표시한 행만 분석에 포함됨</t>
       </text>
     </comment>
     <comment ref="G1" authorId="0" shapeId="0">
       <text>
-        <t>Y로 지정하면 이 작업의 월별합산 결과를 비용구분(판관/제조 등)별로도 나눠서 함께 추출 (공란=기존처럼 구분 없이 합산)</t>
+        <t>Y로 지정하면 이 작업의 월별합산 결과를 전표관리단위(본사/2공장 등)별로도 나눠서 함께 추출 (공란=기존처럼 단위 구분 없이 합산)</t>
       </text>
     </comment>
-    <comment ref="H1" authorId="1" shapeId="0">
+    <comment ref="H1" authorId="0" shapeId="0">
       <text>
-        <t>[스레드 댓글]
-사용 중인 버전의 Excel에서 이 스레드 댓글을 읽을 수 있지만 파일을 이후 버전의 Excel에서 열면 편집 내용이 모두 제거됩니다. 자세한 정보: https://go.microsoft.com/fwlink/?linkid=870924.
-댓글:
-    분리, 통합으로 차변대변 분리해서 표시할지 결정</t>
+        <t>Y로 지정하면 이 작업의 월별합산 결과를 비용구분(판관/제조 등)별로도 나눠서 함께 추출 (공란=기존처럼 구분 없이 합산)</t>
       </text>
     </comment>
   </commentList>
@@ -690,7 +698,7 @@
           <t>StartDate</t>
         </is>
       </c>
-      <c r="B3" s="5" t="n">
+      <c r="B3" s="12" t="n">
         <v>46023</v>
       </c>
       <c r="C3" t="inlineStr">
@@ -705,7 +713,7 @@
           <t>EndDate</t>
         </is>
       </c>
-      <c r="B4" s="5" t="n">
+      <c r="B4" s="12" t="n">
         <v>46387</v>
       </c>
     </row>
@@ -804,15 +812,13 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:N59"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="17"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="9" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="3" max="4"/>
     <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="9" customWidth="1" min="6" max="6"/>
-    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="6" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
     <col width="9" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
@@ -823,72 +829,72 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="7" t="inlineStr">
+      <c r="A1" s="5" t="inlineStr">
         <is>
           <t>계정과목</t>
         </is>
       </c>
-      <c r="B1" s="7" t="inlineStr">
+      <c r="B1" s="5" t="inlineStr">
         <is>
           <t>실행여부</t>
         </is>
       </c>
-      <c r="C1" s="7" t="inlineStr">
+      <c r="C1" s="5" t="inlineStr">
         <is>
           <t>시작일</t>
         </is>
       </c>
-      <c r="D1" s="7" t="inlineStr">
+      <c r="D1" s="5" t="inlineStr">
         <is>
           <t>종료일</t>
         </is>
       </c>
-      <c r="E1" s="7" t="inlineStr">
+      <c r="E1" s="5" t="inlineStr">
         <is>
           <t>샘플링방법</t>
         </is>
       </c>
-      <c r="F1" s="7" t="inlineStr">
+      <c r="F1" s="5" t="inlineStr">
         <is>
           <t>금액타입</t>
         </is>
       </c>
-      <c r="G1" s="7" t="inlineStr">
+      <c r="G1" s="5" t="inlineStr">
         <is>
           <t>샘플크기</t>
         </is>
       </c>
-      <c r="H1" s="7" t="inlineStr">
+      <c r="H1" s="5" t="inlineStr">
         <is>
           <t>통계표사용</t>
         </is>
       </c>
-      <c r="I1" s="7" t="inlineStr">
+      <c r="I1" s="5" t="inlineStr">
         <is>
           <t>신뢰수준</t>
         </is>
       </c>
-      <c r="J1" s="7" t="inlineStr">
+      <c r="J1" s="5" t="inlineStr">
         <is>
           <t>허용왜곡표시</t>
         </is>
       </c>
-      <c r="K1" s="7" t="inlineStr">
+      <c r="K1" s="5" t="inlineStr">
         <is>
           <t>예상왜곡표시</t>
         </is>
       </c>
-      <c r="L1" s="7" t="inlineStr">
+      <c r="L1" s="5" t="inlineStr">
         <is>
           <t>이상거래포함</t>
         </is>
       </c>
-      <c r="M1" s="7" t="inlineStr">
+      <c r="M1" s="5" t="inlineStr">
         <is>
           <t>개별유의금액</t>
         </is>
       </c>
-      <c r="N1" s="7" t="inlineStr">
+      <c r="N1" s="5" t="inlineStr">
         <is>
           <t>비고</t>
         </is>
@@ -905,8 +911,8 @@
           <t>N</t>
         </is>
       </c>
-      <c r="C2" s="9" t="n"/>
-      <c r="D2" s="9" t="n"/>
+      <c r="C2" s="14" t="n"/>
+      <c r="D2" s="14" t="n"/>
       <c r="E2" t="inlineStr">
         <is>
           <t>MUS</t>
@@ -925,11 +931,11 @@
           <t>N</t>
         </is>
       </c>
-      <c r="I2" s="8" t="n">
+      <c r="I2" s="6" t="n">
         <v>0.95</v>
       </c>
-      <c r="J2" s="10" t="n"/>
-      <c r="K2" s="10" t="n">
+      <c r="J2" s="8" t="n"/>
+      <c r="K2" s="8" t="n">
         <v>0</v>
       </c>
       <c r="L2" t="inlineStr">
@@ -937,7 +943,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M2" s="10" t="n"/>
+      <c r="M2" s="8" t="n"/>
       <c r="N2" t="inlineStr">
         <is>
           <t>예시) 매출 실재성 — 차변 MUS 30건</t>
@@ -955,8 +961,8 @@
           <t>N</t>
         </is>
       </c>
-      <c r="C3" s="9" t="n"/>
-      <c r="D3" s="9" t="n"/>
+      <c r="C3" s="14" t="n"/>
+      <c r="D3" s="14" t="n"/>
       <c r="E3" t="inlineStr">
         <is>
           <t>체계적</t>
@@ -975,11 +981,11 @@
           <t>N</t>
         </is>
       </c>
-      <c r="I3" s="8" t="n">
+      <c r="I3" s="6" t="n">
         <v>0.95</v>
       </c>
-      <c r="J3" s="10" t="n"/>
-      <c r="K3" s="10" t="n">
+      <c r="J3" s="8" t="n"/>
+      <c r="K3" s="8" t="n">
         <v>0</v>
       </c>
       <c r="L3" t="inlineStr">
@@ -987,7 +993,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="M3" s="10" t="n"/>
+      <c r="M3" s="8" t="n"/>
       <c r="N3" t="inlineStr">
         <is>
           <t>예시) 출금 증빙 — 대변 체계적 40건</t>
@@ -1005,8 +1011,8 @@
           <t>N</t>
         </is>
       </c>
-      <c r="C4" s="9" t="n"/>
-      <c r="D4" s="9" t="n"/>
+      <c r="C4" s="14" t="n"/>
+      <c r="D4" s="14" t="n"/>
       <c r="E4" t="inlineStr">
         <is>
           <t>MUS</t>
@@ -1022,13 +1028,13 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="I4" s="8" t="n">
+      <c r="I4" s="6" t="n">
         <v>0.95</v>
       </c>
-      <c r="J4" s="10" t="n">
+      <c r="J4" s="8" t="n">
         <v>50000000</v>
       </c>
-      <c r="K4" s="10" t="n">
+      <c r="K4" s="8" t="n">
         <v>0</v>
       </c>
       <c r="L4" t="inlineStr">
@@ -1036,7 +1042,7 @@
           <t>N</t>
         </is>
       </c>
-      <c r="M4" s="10" t="n">
+      <c r="M4" s="8" t="n">
         <v>10000000</v>
       </c>
       <c r="N4" t="inlineStr">
@@ -1046,339 +1052,344 @@
       </c>
     </row>
     <row r="5">
-      <c r="C5" s="9" t="n"/>
-      <c r="D5" s="9" t="n"/>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>상품매출</t>
+        </is>
+      </c>
+      <c r="C5" s="14" t="n"/>
+      <c r="D5" s="14" t="n"/>
     </row>
     <row r="6">
-      <c r="C6" s="9" t="n"/>
-      <c r="D6" s="9" t="n"/>
+      <c r="C6" s="14" t="n"/>
+      <c r="D6" s="14" t="n"/>
     </row>
     <row r="7">
-      <c r="C7" s="9" t="n"/>
-      <c r="D7" s="9" t="n"/>
+      <c r="C7" s="14" t="n"/>
+      <c r="D7" s="14" t="n"/>
     </row>
     <row r="8">
-      <c r="C8" s="9" t="n"/>
-      <c r="D8" s="9" t="n"/>
+      <c r="C8" s="14" t="n"/>
+      <c r="D8" s="14" t="n"/>
     </row>
     <row r="9">
-      <c r="C9" s="9" t="n"/>
-      <c r="D9" s="9" t="n"/>
+      <c r="C9" s="14" t="n"/>
+      <c r="D9" s="14" t="n"/>
     </row>
     <row r="10">
-      <c r="C10" s="9" t="n"/>
-      <c r="D10" s="9" t="n"/>
+      <c r="C10" s="14" t="n"/>
+      <c r="D10" s="14" t="n"/>
     </row>
     <row r="11">
-      <c r="C11" s="9" t="n"/>
-      <c r="D11" s="9" t="n"/>
+      <c r="C11" s="14" t="n"/>
+      <c r="D11" s="14" t="n"/>
     </row>
     <row r="12">
-      <c r="C12" s="9" t="n"/>
-      <c r="D12" s="9" t="n"/>
+      <c r="C12" s="14" t="n"/>
+      <c r="D12" s="14" t="n"/>
     </row>
     <row r="13">
-      <c r="C13" s="9" t="n"/>
-      <c r="D13" s="9" t="n"/>
+      <c r="C13" s="14" t="n"/>
+      <c r="D13" s="14" t="n"/>
     </row>
     <row r="14">
-      <c r="C14" s="9" t="n"/>
-      <c r="D14" s="9" t="n"/>
+      <c r="C14" s="14" t="n"/>
+      <c r="D14" s="14" t="n"/>
     </row>
     <row r="15">
-      <c r="C15" s="9" t="n"/>
-      <c r="D15" s="9" t="n"/>
+      <c r="C15" s="14" t="n"/>
+      <c r="D15" s="14" t="n"/>
     </row>
     <row r="16">
-      <c r="C16" s="9" t="n"/>
-      <c r="D16" s="9" t="n"/>
+      <c r="C16" s="14" t="n"/>
+      <c r="D16" s="14" t="n"/>
     </row>
     <row r="17">
-      <c r="C17" s="9" t="n"/>
-      <c r="D17" s="9" t="n"/>
+      <c r="C17" s="14" t="n"/>
+      <c r="D17" s="14" t="n"/>
     </row>
     <row r="18">
-      <c r="C18" s="9" t="n"/>
-      <c r="D18" s="9" t="n"/>
+      <c r="C18" s="14" t="n"/>
+      <c r="D18" s="14" t="n"/>
     </row>
     <row r="19">
-      <c r="C19" s="9" t="n"/>
-      <c r="D19" s="9" t="n"/>
+      <c r="C19" s="14" t="n"/>
+      <c r="D19" s="14" t="n"/>
     </row>
     <row r="20">
-      <c r="C20" s="9" t="n"/>
-      <c r="D20" s="9" t="n"/>
+      <c r="C20" s="14" t="n"/>
+      <c r="D20" s="14" t="n"/>
     </row>
     <row r="21">
-      <c r="C21" s="9" t="n"/>
-      <c r="D21" s="9" t="n"/>
+      <c r="C21" s="14" t="n"/>
+      <c r="D21" s="14" t="n"/>
     </row>
     <row r="22">
-      <c r="C22" s="9" t="n"/>
-      <c r="D22" s="9" t="n"/>
+      <c r="C22" s="14" t="n"/>
+      <c r="D22" s="14" t="n"/>
     </row>
     <row r="23">
-      <c r="C23" s="9" t="n"/>
-      <c r="D23" s="9" t="n"/>
+      <c r="C23" s="14" t="n"/>
+      <c r="D23" s="14" t="n"/>
     </row>
     <row r="24">
-      <c r="C24" s="9" t="n"/>
-      <c r="D24" s="9" t="n"/>
+      <c r="C24" s="14" t="n"/>
+      <c r="D24" s="14" t="n"/>
     </row>
     <row r="25">
-      <c r="C25" s="9" t="n"/>
-      <c r="D25" s="9" t="n"/>
+      <c r="C25" s="14" t="n"/>
+      <c r="D25" s="14" t="n"/>
     </row>
     <row r="26">
-      <c r="C26" s="9" t="n"/>
-      <c r="D26" s="9" t="n"/>
+      <c r="C26" s="14" t="n"/>
+      <c r="D26" s="14" t="n"/>
     </row>
     <row r="27">
-      <c r="C27" s="9" t="n"/>
-      <c r="D27" s="9" t="n"/>
+      <c r="C27" s="14" t="n"/>
+      <c r="D27" s="14" t="n"/>
     </row>
     <row r="28">
-      <c r="C28" s="9" t="n"/>
-      <c r="D28" s="9" t="n"/>
+      <c r="C28" s="14" t="n"/>
+      <c r="D28" s="14" t="n"/>
     </row>
     <row r="29">
-      <c r="C29" s="9" t="n"/>
-      <c r="D29" s="9" t="n"/>
+      <c r="C29" s="14" t="n"/>
+      <c r="D29" s="14" t="n"/>
     </row>
     <row r="30">
-      <c r="C30" s="9" t="n"/>
-      <c r="D30" s="9" t="n"/>
+      <c r="C30" s="14" t="n"/>
+      <c r="D30" s="14" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="11" t="inlineStr">
+      <c r="A31" s="9" t="inlineStr">
         <is>
           <t>■ 15번 감사샘플링 작성 안내 (이 안내 행들은 실행여부가 비어 있어 분석에 읽히지 않음 — 지우지 말고 위쪽 행에 계정 입력)</t>
         </is>
       </c>
-      <c r="C31" s="9" t="n"/>
-      <c r="D31" s="9" t="n"/>
+      <c r="C31" s="14" t="n"/>
+      <c r="D31" s="14" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="12" t="inlineStr">
+      <c r="A32" s="10" t="inlineStr">
         <is>
           <t>[기본 항목]</t>
         </is>
       </c>
-      <c r="C32" s="9" t="n"/>
-      <c r="D32" s="9" t="n"/>
+      <c r="C32" s="14" t="n"/>
+      <c r="D32" s="14" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="13" t="inlineStr">
+      <c r="A33" s="11" t="inlineStr">
         <is>
           <t>· 실행여부: Y(또는 O)인 행만 실행.  · 시작일/종료일: 비우면 분개장 전체 기간.</t>
         </is>
       </c>
-      <c r="C33" s="9" t="n"/>
-      <c r="D33" s="9" t="n"/>
+      <c r="C33" s="14" t="n"/>
+      <c r="D33" s="14" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="13" t="inlineStr">
+      <c r="A34" s="11" t="inlineStr">
         <is>
           <t>· 샘플링방법: MUS / 체계적 / 무작위 / 금액상위 (빈칸 = MUS).</t>
         </is>
       </c>
-      <c r="C34" s="9" t="n"/>
-      <c r="D34" s="9" t="n"/>
+      <c r="C34" s="14" t="n"/>
+      <c r="D34" s="14" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="13" t="inlineStr">
+      <c r="A35" s="11" t="inlineStr">
         <is>
           <t>· 금액타입: 차변 / 대변 / both (빈칸·그 외 값 = both). 결과시트명은 계정명_차 / _대 / _양.</t>
         </is>
       </c>
-      <c r="C35" s="9" t="n"/>
-      <c r="D35" s="9" t="n"/>
+      <c r="C35" s="14" t="n"/>
+      <c r="D35" s="14" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="12" t="inlineStr">
+      <c r="A36" s="10" t="inlineStr">
         <is>
           <t>[샘플크기 — 통계표사용에 따라 결정]</t>
         </is>
       </c>
-      <c r="C36" s="9" t="n"/>
-      <c r="D36" s="9" t="n"/>
+      <c r="C36" s="14" t="n"/>
+      <c r="D36" s="14" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="13" t="inlineStr">
+      <c r="A37" s="11" t="inlineStr">
         <is>
           <t>· 통계표사용 = N(또는 빈칸): 샘플크기 칸의 입력값대로 추출 (빈칸 = 30건). 신뢰수준·허용/예상왜곡표시는 무시됨.</t>
         </is>
       </c>
-      <c r="C37" s="9" t="n"/>
-      <c r="D37" s="9" t="n"/>
+      <c r="C37" s="14" t="n"/>
+      <c r="D37" s="14" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="13" t="inlineStr">
+      <c r="A38" s="11" t="inlineStr">
         <is>
           <t>· 통계표사용 = Y: 샘플크기 = 모집단금액 × 신뢰계수 ÷ (허용왜곡표시 − 예상왜곡표시 × 확장계수) 로 자동 계산, 샘플크기 칸 입력값은 무시됨.</t>
         </is>
       </c>
-      <c r="C38" s="9" t="n"/>
-      <c r="D38" s="9" t="n"/>
+      <c r="C38" s="14" t="n"/>
+      <c r="D38" s="14" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="13" t="inlineStr">
+      <c r="A39" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">    - 신뢰계수/확장계수: 90% = 2.31/1.5, 95% = 3.00/1.6, 99% = 4.61/1.9 (모집단금액은 개별유의금액 전수분을 뺀 금액).</t>
         </is>
       </c>
-      <c r="C39" s="9" t="n"/>
-      <c r="D39" s="9" t="n"/>
+      <c r="C39" s="14" t="n"/>
+      <c r="D39" s="14" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="13" t="inlineStr">
+      <c r="A40" s="11" t="inlineStr">
         <is>
           <t>· 신뢰수준: 0.95 또는 95 둘 다 가능 (빈칸 = 0.95). 90/95/99% 중 가까운 값 적용.</t>
         </is>
       </c>
-      <c r="C40" s="9" t="n"/>
-      <c r="D40" s="9" t="n"/>
+      <c r="C40" s="14" t="n"/>
+      <c r="D40" s="14" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" s="13" t="inlineStr">
+      <c r="A41" s="11" t="inlineStr">
         <is>
           <t>· 허용왜곡표시: 통계표사용 = Y이면 필수(예: 수행중요성). 비우면 해당 계정은 샘플 미추출 → 샘플링조건 시트 결과시트 "미추출" + 비고에 사유 표시.</t>
         </is>
       </c>
-      <c r="C41" s="9" t="n"/>
-      <c r="D41" s="9" t="n"/>
+      <c r="C41" s="14" t="n"/>
+      <c r="D41" s="14" t="n"/>
     </row>
     <row r="42">
-      <c r="A42" s="13" t="inlineStr">
+      <c r="A42" s="11" t="inlineStr">
         <is>
           <t>· 예상왜곡표시: 비워도 됨(빈칸 = 0). 0이면 샘플크기가 가장 작게 나오고, 전기 왜곡표시 등 오류 위험이 있으면 금액을 넣어 보수적으로(샘플 증가).</t>
         </is>
       </c>
-      <c r="C42" s="9" t="n"/>
-      <c r="D42" s="9" t="n"/>
+      <c r="C42" s="14" t="n"/>
+      <c r="D42" s="14" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="13" t="inlineStr">
+      <c r="A43" s="11" t="inlineStr">
         <is>
           <t xml:space="preserve">    - 예상왜곡표시 × 확장계수 ≥ 허용왜곡표시 이면 계산 불가 → 해당 계정 건너뛰고 비고에 사유 표시.</t>
         </is>
       </c>
-      <c r="C43" s="9" t="n"/>
-      <c r="D43" s="9" t="n"/>
+      <c r="C43" s="14" t="n"/>
+      <c r="D43" s="14" t="n"/>
     </row>
     <row r="44">
-      <c r="A44" s="12" t="inlineStr">
+      <c r="A44" s="10" t="inlineStr">
         <is>
           <t>[금액 입력 형식 — 허용왜곡표시·예상왜곡표시·개별유의금액]</t>
         </is>
       </c>
-      <c r="C44" s="9" t="n"/>
-      <c r="D44" s="9" t="n"/>
+      <c r="C44" s="14" t="n"/>
+      <c r="D44" s="14" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="13" t="inlineStr">
+      <c r="A45" s="11" t="inlineStr">
         <is>
           <t>· 원 단위 숫자로 입력: 500000000 또는 500,000,000 (엑셀 숫자 셀 OK).</t>
         </is>
       </c>
-      <c r="C45" s="9" t="n"/>
-      <c r="D45" s="9" t="n"/>
+      <c r="C45" s="14" t="n"/>
+      <c r="D45" s="14" t="n"/>
     </row>
     <row r="46">
-      <c r="A46" s="13" t="inlineStr">
+      <c r="A46" s="11" t="inlineStr">
         <is>
           <t>· "5억", "500,000,000원"처럼 글자가 섞이면 빈칸으로 처리됨. "5%", 0.05 같은 비율 입력 금지(5원·0.05원으로 읽힘).</t>
         </is>
       </c>
-      <c r="C46" s="9" t="n"/>
-      <c r="D46" s="9" t="n"/>
+      <c r="C46" s="14" t="n"/>
+      <c r="D46" s="14" t="n"/>
     </row>
     <row r="47">
-      <c r="A47" s="12" t="inlineStr">
+      <c r="A47" s="10" t="inlineStr">
         <is>
           <t>[추가 옵션]</t>
         </is>
       </c>
-      <c r="C47" s="9" t="n"/>
-      <c r="D47" s="9" t="n"/>
+      <c r="C47" s="14" t="n"/>
+      <c r="D47" s="14" t="n"/>
     </row>
     <row r="48">
-      <c r="A48" s="13" t="inlineStr">
+      <c r="A48" s="11" t="inlineStr">
         <is>
           <t>· 개별유의금액: 이 금액 이상인 줄은 전수 추출(샘플크기와 별도로 추가). 빈칸 = 전수 없음.</t>
         </is>
       </c>
-      <c r="C48" s="9" t="n"/>
-      <c r="D48" s="9" t="n"/>
+      <c r="C48" s="14" t="n"/>
+      <c r="D48" s="14" t="n"/>
     </row>
     <row r="49">
-      <c r="A49" s="13" t="inlineStr">
+      <c r="A49" s="11" t="inlineStr">
         <is>
           <t>· 이상거래포함 = Y: 최대값 + Z-score 3 이상 거래를 샘플크기의 20%까지 먼저 포함(샘플크기 안에 포함됨).</t>
         </is>
       </c>
-      <c r="C49" s="9" t="n"/>
-      <c r="D49" s="9" t="n"/>
+      <c r="C49" s="14" t="n"/>
+      <c r="D49" s="14" t="n"/>
     </row>
     <row r="50">
-      <c r="A50" s="12" t="inlineStr">
+      <c r="A50" s="10" t="inlineStr">
         <is>
           <t>[결과 확인]</t>
         </is>
       </c>
-      <c r="C50" s="9" t="n"/>
-      <c r="D50" s="9" t="n"/>
+      <c r="C50" s="14" t="n"/>
+      <c r="D50" s="14" t="n"/>
     </row>
     <row r="51">
-      <c r="A51" s="13" t="inlineStr">
+      <c r="A51" s="11" t="inlineStr">
         <is>
           <t>· 샘플링조건 시트: 계정별 모집단·원장 대사·샘플크기 근거·추출조건 요약. 샘플 시트가 안 나오면 이 시트의 결과시트·비고 열부터 확인.</t>
         </is>
       </c>
-      <c r="C51" s="9" t="n"/>
-      <c r="D51" s="9" t="n"/>
+      <c r="C51" s="14" t="n"/>
+      <c r="D51" s="14" t="n"/>
     </row>
     <row r="52">
-      <c r="A52" s="13" t="inlineStr">
+      <c r="A52" s="11" t="inlineStr">
         <is>
           <t>· 샘플 단위는 해당 계정의 전표 "줄". 같은 전표의 상대계정 줄은 뽑지 않고 상대계정 열에 참고로만 표시.</t>
         </is>
       </c>
-      <c r="C52" s="9" t="n"/>
-      <c r="D52" s="9" t="n"/>
+      <c r="C52" s="14" t="n"/>
+      <c r="D52" s="14" t="n"/>
     </row>
     <row r="53">
-      <c r="A53" s="13" t="inlineStr">
+      <c r="A53" s="11" t="inlineStr">
         <is>
           <t>· 시드 42 고정 → 같은 조건으로 재실행하면 같은 샘플(조서 재현성). 증빙종류~확인자 열은 감사인이 직접 기재.</t>
         </is>
       </c>
-      <c r="C53" s="9" t="n"/>
-      <c r="D53" s="9" t="n"/>
+      <c r="C53" s="14" t="n"/>
+      <c r="D53" s="14" t="n"/>
     </row>
     <row r="54">
-      <c r="C54" s="9" t="n"/>
-      <c r="D54" s="9" t="n"/>
+      <c r="C54" s="14" t="n"/>
+      <c r="D54" s="14" t="n"/>
     </row>
     <row r="55">
-      <c r="C55" s="9" t="n"/>
-      <c r="D55" s="9" t="n"/>
+      <c r="C55" s="14" t="n"/>
+      <c r="D55" s="14" t="n"/>
     </row>
     <row r="56">
-      <c r="C56" s="9" t="n"/>
-      <c r="D56" s="9" t="n"/>
+      <c r="C56" s="14" t="n"/>
+      <c r="D56" s="14" t="n"/>
     </row>
     <row r="57">
-      <c r="C57" s="9" t="n"/>
-      <c r="D57" s="9" t="n"/>
+      <c r="C57" s="14" t="n"/>
+      <c r="D57" s="14" t="n"/>
     </row>
     <row r="58">
-      <c r="C58" s="9" t="n"/>
-      <c r="D58" s="9" t="n"/>
+      <c r="C58" s="14" t="n"/>
+      <c r="D58" s="14" t="n"/>
     </row>
     <row r="59">
-      <c r="C59" s="9" t="n"/>
-      <c r="D59" s="9" t="n"/>
+      <c r="C59" s="14" t="n"/>
+      <c r="D59" s="14" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="3">
@@ -1402,13 +1413,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="17"/>
   <cols>
     <col width="27.75" customWidth="1" min="1" max="1"/>
-    <col width="26.9140625" bestFit="1" customWidth="1" min="2" max="2"/>
-    <col width="35.25" bestFit="1" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="5" max="7"/>
+    <col width="26.9140625" customWidth="1" min="2" max="2"/>
+    <col width="35.25" customWidth="1" min="3" max="3"/>
+    <col width="25" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1429,25 +1441,30 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
+          <t>적요</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
           <t>금액열</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>실행여부</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>관리단위</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>비용구분</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>표시방식</t>
         </is>
@@ -1456,7 +1473,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>※ 사용법: 작업명(자유기재) / 계정과목·거래처명은 콤마로 여러 개 가능 / 금액열: 차변·대변·both / 실행여부 Y인 행만 처리됨</t>
+          <t>※ 사용법: 작업명(자유기재) / 계정과목·거래처명·적요는 콤마로 여러 개 가능 / 적요 기재 시 적요 조건도 추가(공란=조건 없음) / 금액열: 차변·대변·both / 실행여부 Y인 행만 처리됨</t>
         </is>
       </c>
     </row>
@@ -1476,12 +1493,12 @@
           <t>리브퓨어(미국본사)</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>대변</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -1503,12 +1520,12 @@
           <t>리브퓨어(태국지사)</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>대변</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -1530,12 +1547,12 @@
           <t>코스맥스엔비티 주식회사</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>차변</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -1557,12 +1574,12 @@
           <t>리브퓨어(미국본사)</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>차변</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -1584,17 +1601,17 @@
           <t>코스맥스엔비티 주식회사</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>차변</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
         <is>
           <t>분리</t>
         </is>
@@ -1616,17 +1633,17 @@
           <t>리브퓨어(미국본사)</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="E8" t="inlineStr">
         <is>
           <t>차변</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
         <is>
           <t>분리</t>
         </is>
@@ -1648,12 +1665,12 @@
           <t>리브퓨어(미국본사)</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="E9" t="inlineStr">
         <is>
           <t>차변</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="F9" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -1675,12 +1692,12 @@
           <t>(주)콘코디아테크널러지</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="E10" t="inlineStr">
         <is>
           <t>차변</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="F10" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -1882,7 +1899,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="17"/>
   <cols>
     <col width="16.25" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -1950,6 +1967,50 @@
         </is>
       </c>
       <c r="D3" t="inlineStr">
+        <is>
+          <t>분리</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>잡이익</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>대변</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>분리</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>제품운송비</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>차변</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
         <is>
           <t>분리</t>
         </is>
@@ -2986,68 +3047,65 @@
     <col width="18" bestFit="1" customWidth="1" min="1" max="1"/>
     <col width="9" customWidth="1" min="2" max="2"/>
     <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="9" customWidth="1" min="4" max="4"/>
-    <col width="9" customWidth="1" min="5" max="5"/>
-    <col width="9" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="4" max="6"/>
     <col width="7" customWidth="1" min="7" max="7"/>
     <col width="8" customWidth="1" min="8" max="8"/>
-    <col width="7" customWidth="1" min="9" max="9"/>
-    <col width="7" customWidth="1" min="10" max="10"/>
+    <col width="7" customWidth="1" min="9" max="10"/>
     <col width="50" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="7" t="inlineStr">
+      <c r="A1" s="5" t="inlineStr">
         <is>
           <t>계정과목</t>
         </is>
       </c>
-      <c r="B1" s="7" t="inlineStr">
+      <c r="B1" s="5" t="inlineStr">
         <is>
           <t>실행여부</t>
         </is>
       </c>
-      <c r="C1" s="7" t="inlineStr">
+      <c r="C1" s="5" t="inlineStr">
         <is>
           <t>샘플링비율</t>
         </is>
       </c>
-      <c r="D1" s="7" t="inlineStr">
+      <c r="D1" s="5" t="inlineStr">
         <is>
           <t>최소건수</t>
         </is>
       </c>
-      <c r="E1" s="7" t="inlineStr">
+      <c r="E1" s="5" t="inlineStr">
         <is>
           <t>최대건수</t>
         </is>
       </c>
-      <c r="F1" s="7" t="inlineStr">
+      <c r="F1" s="5" t="inlineStr">
         <is>
           <t>금액상위</t>
         </is>
       </c>
-      <c r="G1" s="7" t="inlineStr">
+      <c r="G1" s="5" t="inlineStr">
         <is>
           <t>최신</t>
         </is>
       </c>
-      <c r="H1" s="7" t="inlineStr">
+      <c r="H1" s="5" t="inlineStr">
         <is>
           <t>이상치</t>
         </is>
       </c>
-      <c r="I1" s="7" t="inlineStr">
+      <c r="I1" s="5" t="inlineStr">
         <is>
           <t>월별</t>
         </is>
       </c>
-      <c r="J1" s="7" t="inlineStr">
+      <c r="J1" s="5" t="inlineStr">
         <is>
           <t>랜덤</t>
         </is>
       </c>
-      <c r="K1" s="7" t="inlineStr">
+      <c r="K1" s="5" t="inlineStr">
         <is>
           <t>중점검토사항</t>
         </is>
@@ -3064,7 +3122,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="C2" s="8" t="n">
+      <c r="C2" s="6" t="n">
         <v>0.05</v>
       </c>
       <c r="D2" t="n">
@@ -3073,19 +3131,19 @@
       <c r="E2" t="n">
         <v>150</v>
       </c>
-      <c r="F2" s="8" t="n">
+      <c r="F2" s="6" t="n">
         <v>0.3</v>
       </c>
-      <c r="G2" s="8" t="n">
+      <c r="G2" s="6" t="n">
         <v>0.2</v>
       </c>
-      <c r="H2" s="8" t="n">
+      <c r="H2" s="6" t="n">
         <v>0.1</v>
       </c>
-      <c r="I2" s="8" t="n">
+      <c r="I2" s="6" t="n">
         <v>0.3</v>
       </c>
-      <c r="J2" s="8" t="n">
+      <c r="J2" s="6" t="n">
         <v>0.1</v>
       </c>
     </row>
@@ -5169,19 +5227,19 @@
       </c>
     </row>
     <row r="2">
-      <c r="C2" s="6" t="n"/>
+      <c r="C2" s="13" t="n"/>
     </row>
     <row r="3">
-      <c r="C3" s="6" t="n"/>
+      <c r="C3" s="13" t="n"/>
     </row>
     <row r="4">
-      <c r="C4" s="6" t="n"/>
+      <c r="C4" s="13" t="n"/>
     </row>
     <row r="5">
-      <c r="C5" s="6" t="n"/>
+      <c r="C5" s="13" t="n"/>
     </row>
     <row r="6">
-      <c r="C6" s="6" t="n"/>
+      <c r="C6" s="13" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>